<commit_message>
Add test data and 1 x n vectorization for rows and columns.
</commit_message>
<xml_diff>
--- a/tests/data/parameters.xlsx
+++ b/tests/data/parameters.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="33">
   <si>
     <t>hours</t>
   </si>
@@ -35,6 +35,9 @@
     <t>7:00 am - 8:00 pm</t>
   </si>
   <si>
+    <t>jumps</t>
+  </si>
+  <si>
     <t>prices</t>
   </si>
   <si>
@@ -44,6 +47,9 @@
     <t>Tuesday</t>
   </si>
   <si>
+    <t>over</t>
+  </si>
+  <si>
     <t>title</t>
   </si>
   <si>
@@ -53,6 +59,18 @@
     <t>Wednesday</t>
   </si>
   <si>
+    <t>the</t>
+  </si>
+  <si>
+    <t>quick</t>
+  </si>
+  <si>
+    <t>brown</t>
+  </si>
+  <si>
+    <t>fox</t>
+  </si>
+  <si>
     <t>hours_list</t>
   </si>
   <si>
@@ -62,7 +80,25 @@
     <t>Thursday</t>
   </si>
   <si>
+    <t>lazy</t>
+  </si>
+  <si>
+    <t>h_vector</t>
+  </si>
+  <si>
+    <t>[H5:K5]</t>
+  </si>
+  <si>
     <t>Friday</t>
+  </si>
+  <si>
+    <t>dog</t>
+  </si>
+  <si>
+    <t>v_vector</t>
+  </si>
+  <si>
+    <t>[H3:H7]</t>
   </si>
   <si>
     <t>Saturday</t>
@@ -375,77 +411,113 @@
       <c r="E3" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="H3" s="3" t="s">
+        <v>4</v>
+      </c>
       <c r="L3" s="1"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>3</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>8</v>
       </c>
       <c r="M4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>3</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="M5" s="1"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>3</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="M6" s="1"/>
     </row>
     <row r="7">
+      <c r="A7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>21</v>
+      </c>
       <c r="D7" s="1" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>3</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>23</v>
       </c>
       <c r="M7" s="1"/>
     </row>
     <row r="8">
+      <c r="A8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>25</v>
+      </c>
       <c r="D8" s="1" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="M8" s="1"/>
     </row>
     <row r="9">
       <c r="D9" s="1" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -1449,7 +1521,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="B1" s="4">
         <v>3.25</v>
@@ -1457,7 +1529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="B2" s="4">
         <v>4.0</v>
@@ -1465,7 +1537,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="B3" s="3">
         <v>8.25</v>

</xml_diff>